<commit_message>
feat(qa): replace placeholder scenarios with unique feature-specific test descriptions and regenerate all Excel reports
</commit_message>
<xml_diff>
--- a/tests/reports/DentNova_Full_Test_Report.xlsx
+++ b/tests/reports/DentNova_Full_Test_Report.xlsx
@@ -889,7 +889,7 @@
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Generated: 2026-07-14 20:40:11 | Tester: DentNova QA Automation</t>
+          <t>Generated: 2026-07-25 23:05:16 | Tester: DentNova QA Automation</t>
         </is>
       </c>
     </row>
@@ -1480,7 +1480,7 @@
       </c>
       <c r="R2" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S2" s="6" t="inlineStr">
@@ -1575,7 +1575,7 @@
       </c>
       <c r="R3" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S3" s="6" t="inlineStr">
@@ -1670,7 +1670,7 @@
       </c>
       <c r="R4" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S4" s="6" t="inlineStr">
@@ -1765,7 +1765,7 @@
       </c>
       <c r="R5" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S5" s="6" t="inlineStr">
@@ -1860,7 +1860,7 @@
       </c>
       <c r="R6" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S6" s="6" t="inlineStr">
@@ -2392,7 +2392,7 @@
       </c>
       <c r="R12" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S12" s="6" t="inlineStr">
@@ -2487,7 +2487,7 @@
       </c>
       <c r="R13" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S13" s="6" t="inlineStr">
@@ -2584,7 +2584,7 @@
       </c>
       <c r="R14" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S14" s="6" t="inlineStr">
@@ -2678,7 +2678,7 @@
       </c>
       <c r="R15" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S15" s="6" t="inlineStr">
@@ -2773,7 +2773,7 @@
       </c>
       <c r="R16" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S16" s="6" t="inlineStr">
@@ -2868,7 +2868,7 @@
       </c>
       <c r="R17" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S17" s="6" t="inlineStr">
@@ -2963,7 +2963,7 @@
       </c>
       <c r="R18" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S18" s="6" t="inlineStr">
@@ -3058,7 +3058,7 @@
       </c>
       <c r="R19" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S19" s="6" t="inlineStr">
@@ -3152,7 +3152,7 @@
       </c>
       <c r="R20" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S20" s="6" t="inlineStr">
@@ -3247,7 +3247,7 @@
       </c>
       <c r="R21" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S21" s="6" t="inlineStr">
@@ -3438,7 +3438,7 @@
       </c>
       <c r="R23" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S23" s="6" t="inlineStr">
@@ -3533,7 +3533,7 @@
       </c>
       <c r="R24" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S24" s="6" t="inlineStr">
@@ -3629,7 +3629,7 @@
       </c>
       <c r="R25" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S25" s="6" t="inlineStr">
@@ -7798,7 +7798,7 @@
       </c>
       <c r="R72" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S72" s="6" t="inlineStr">
@@ -8744,7 +8744,7 @@
       </c>
       <c r="R82" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S82" s="6" t="inlineStr">
@@ -10049,7 +10049,7 @@
       </c>
       <c r="R97" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S97" s="6" t="inlineStr">
@@ -10618,7 +10618,7 @@
       </c>
       <c r="R103" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S103" s="6" t="inlineStr">
@@ -11407,7 +11407,7 @@
       </c>
       <c r="R112" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S112" s="6" t="inlineStr">
@@ -11783,7 +11783,7 @@
       </c>
       <c r="R116" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S116" s="6" t="inlineStr">
@@ -12743,7 +12743,7 @@
       </c>
       <c r="R127" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S127" s="6" t="inlineStr">
@@ -13214,7 +13214,7 @@
       </c>
       <c r="R132" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S132" s="6" t="inlineStr">
@@ -13657,7 +13657,7 @@
       </c>
       <c r="R137" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S137" s="6" t="inlineStr">
@@ -14037,7 +14037,7 @@
       </c>
       <c r="R141" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S141" s="6" t="inlineStr">
@@ -14131,7 +14131,7 @@
       </c>
       <c r="R142" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S142" s="6" t="inlineStr">
@@ -14793,7 +14793,7 @@
       </c>
       <c r="R149" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S149" s="6" t="inlineStr">
@@ -15202,7 +15202,7 @@
       <c r="Q2" s="6" t="inlineStr"/>
       <c r="R2" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S2" s="6" t="inlineStr">
@@ -15296,7 +15296,7 @@
       <c r="Q3" s="6" t="inlineStr"/>
       <c r="R3" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S3" s="6" t="inlineStr">
@@ -15391,7 +15391,7 @@
       <c r="Q4" s="6" t="inlineStr"/>
       <c r="R4" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S4" s="6" t="inlineStr">
@@ -15485,7 +15485,7 @@
       <c r="Q5" s="6" t="inlineStr"/>
       <c r="R5" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S5" s="6" t="inlineStr">
@@ -15579,7 +15579,7 @@
       <c r="Q6" s="6" t="inlineStr"/>
       <c r="R6" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S6" s="6" t="inlineStr">
@@ -15675,7 +15675,7 @@
       <c r="Q7" s="6" t="inlineStr"/>
       <c r="R7" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S7" s="6" t="inlineStr">
@@ -15770,7 +15770,7 @@
       <c r="Q8" s="6" t="inlineStr"/>
       <c r="R8" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S8" s="6" t="inlineStr">
@@ -15865,7 +15865,7 @@
       <c r="Q9" s="6" t="inlineStr"/>
       <c r="R9" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S9" s="6" t="inlineStr">
@@ -15959,7 +15959,7 @@
       <c r="Q10" s="6" t="inlineStr"/>
       <c r="R10" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S10" s="6" t="inlineStr">
@@ -16053,7 +16053,7 @@
       <c r="Q11" s="6" t="inlineStr"/>
       <c r="R11" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S11" s="6" t="inlineStr">
@@ -16147,7 +16147,7 @@
       <c r="Q12" s="6" t="inlineStr"/>
       <c r="R12" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S12" s="6" t="inlineStr">
@@ -16242,7 +16242,7 @@
       <c r="Q13" s="6" t="inlineStr"/>
       <c r="R13" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S13" s="6" t="inlineStr">
@@ -16337,7 +16337,7 @@
       <c r="Q14" s="6" t="inlineStr"/>
       <c r="R14" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S14" s="6" t="inlineStr">
@@ -16433,7 +16433,7 @@
       <c r="Q15" s="6" t="inlineStr"/>
       <c r="R15" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S15" s="6" t="inlineStr">
@@ -16527,7 +16527,7 @@
       <c r="Q16" s="6" t="inlineStr"/>
       <c r="R16" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S16" s="6" t="inlineStr">
@@ -16621,7 +16621,7 @@
       <c r="Q17" s="6" t="inlineStr"/>
       <c r="R17" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S17" s="6" t="inlineStr">
@@ -16716,7 +16716,7 @@
       <c r="Q18" s="6" t="inlineStr"/>
       <c r="R18" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S18" s="6" t="inlineStr">
@@ -16810,7 +16810,7 @@
       <c r="Q19" s="6" t="inlineStr"/>
       <c r="R19" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S19" s="6" t="inlineStr">
@@ -16904,7 +16904,7 @@
       <c r="Q20" s="6" t="inlineStr"/>
       <c r="R20" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S20" s="6" t="inlineStr">
@@ -16998,7 +16998,7 @@
       <c r="Q21" s="6" t="inlineStr"/>
       <c r="R21" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S21" s="6" t="inlineStr">
@@ -17092,7 +17092,7 @@
       <c r="Q22" s="6" t="inlineStr"/>
       <c r="R22" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S22" s="6" t="inlineStr">
@@ -17186,7 +17186,7 @@
       <c r="Q23" s="6" t="inlineStr"/>
       <c r="R23" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S23" s="6" t="inlineStr">
@@ -17280,7 +17280,7 @@
       <c r="Q24" s="6" t="inlineStr"/>
       <c r="R24" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S24" s="6" t="inlineStr">
@@ -17374,7 +17374,7 @@
       <c r="Q25" s="6" t="inlineStr"/>
       <c r="R25" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S25" s="6" t="inlineStr">
@@ -17469,7 +17469,7 @@
       <c r="Q26" s="6" t="inlineStr"/>
       <c r="R26" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S26" s="6" t="inlineStr">
@@ -17563,7 +17563,7 @@
       <c r="Q27" s="6" t="inlineStr"/>
       <c r="R27" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S27" s="6" t="inlineStr">
@@ -17657,7 +17657,7 @@
       <c r="Q28" s="6" t="inlineStr"/>
       <c r="R28" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S28" s="6" t="inlineStr">
@@ -17751,7 +17751,7 @@
       <c r="Q29" s="6" t="inlineStr"/>
       <c r="R29" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S29" s="6" t="inlineStr">
@@ -17846,7 +17846,7 @@
       <c r="Q30" s="6" t="inlineStr"/>
       <c r="R30" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S30" s="6" t="inlineStr">
@@ -17940,7 +17940,7 @@
       <c r="Q31" s="6" t="inlineStr"/>
       <c r="R31" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S31" s="6" t="inlineStr">
@@ -18035,7 +18035,7 @@
       <c r="Q32" s="6" t="inlineStr"/>
       <c r="R32" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S32" s="6" t="inlineStr">
@@ -18129,7 +18129,7 @@
       <c r="Q33" s="6" t="inlineStr"/>
       <c r="R33" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S33" s="6" t="inlineStr">
@@ -18223,7 +18223,7 @@
       <c r="Q34" s="6" t="inlineStr"/>
       <c r="R34" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S34" s="6" t="inlineStr">
@@ -18318,7 +18318,7 @@
       <c r="Q35" s="6" t="inlineStr"/>
       <c r="R35" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S35" s="6" t="inlineStr">
@@ -18412,7 +18412,7 @@
       <c r="Q36" s="6" t="inlineStr"/>
       <c r="R36" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S36" s="6" t="inlineStr">
@@ -18506,7 +18506,7 @@
       <c r="Q37" s="6" t="inlineStr"/>
       <c r="R37" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S37" s="6" t="inlineStr">
@@ -18602,7 +18602,7 @@
       <c r="Q38" s="6" t="inlineStr"/>
       <c r="R38" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S38" s="6" t="inlineStr">
@@ -18696,7 +18696,7 @@
       <c r="Q39" s="6" t="inlineStr"/>
       <c r="R39" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S39" s="6" t="inlineStr">
@@ -18790,7 +18790,7 @@
       <c r="Q40" s="6" t="inlineStr"/>
       <c r="R40" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S40" s="6" t="inlineStr">
@@ -18884,7 +18884,7 @@
       <c r="Q41" s="6" t="inlineStr"/>
       <c r="R41" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S41" s="6" t="inlineStr">
@@ -18979,7 +18979,7 @@
       <c r="Q42" s="6" t="inlineStr"/>
       <c r="R42" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S42" s="6" t="inlineStr">
@@ -19073,7 +19073,7 @@
       <c r="Q43" s="6" t="inlineStr"/>
       <c r="R43" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S43" s="6" t="inlineStr">
@@ -19167,7 +19167,7 @@
       <c r="Q44" s="6" t="inlineStr"/>
       <c r="R44" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S44" s="6" t="inlineStr">
@@ -19262,7 +19262,7 @@
       <c r="Q45" s="6" t="inlineStr"/>
       <c r="R45" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S45" s="6" t="inlineStr">
@@ -19356,7 +19356,7 @@
       <c r="Q46" s="6" t="inlineStr"/>
       <c r="R46" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S46" s="6" t="inlineStr">
@@ -19450,7 +19450,7 @@
       <c r="Q47" s="6" t="inlineStr"/>
       <c r="R47" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S47" s="6" t="inlineStr">
@@ -19544,7 +19544,7 @@
       <c r="Q48" s="6" t="inlineStr"/>
       <c r="R48" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S48" s="6" t="inlineStr">
@@ -19638,7 +19638,7 @@
       <c r="Q49" s="6" t="inlineStr"/>
       <c r="R49" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S49" s="6" t="inlineStr">
@@ -19732,7 +19732,7 @@
       <c r="Q50" s="6" t="inlineStr"/>
       <c r="R50" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S50" s="6" t="inlineStr">
@@ -19826,7 +19826,7 @@
       <c r="Q51" s="6" t="inlineStr"/>
       <c r="R51" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S51" s="6" t="inlineStr">
@@ -19921,7 +19921,7 @@
       <c r="Q52" s="6" t="inlineStr"/>
       <c r="R52" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S52" s="6" t="inlineStr">
@@ -20015,7 +20015,7 @@
       <c r="Q53" s="6" t="inlineStr"/>
       <c r="R53" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S53" s="6" t="inlineStr">
@@ -20109,7 +20109,7 @@
       <c r="Q54" s="6" t="inlineStr"/>
       <c r="R54" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S54" s="6" t="inlineStr">
@@ -20205,7 +20205,7 @@
       <c r="Q55" s="6" t="inlineStr"/>
       <c r="R55" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S55" s="6" t="inlineStr">
@@ -20299,7 +20299,7 @@
       <c r="Q56" s="6" t="inlineStr"/>
       <c r="R56" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S56" s="6" t="inlineStr">
@@ -20394,7 +20394,7 @@
       <c r="Q57" s="6" t="inlineStr"/>
       <c r="R57" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S57" s="6" t="inlineStr">
@@ -20489,7 +20489,7 @@
       <c r="Q58" s="6" t="inlineStr"/>
       <c r="R58" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S58" s="6" t="inlineStr">
@@ -20584,7 +20584,7 @@
       <c r="Q59" s="6" t="inlineStr"/>
       <c r="R59" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S59" s="6" t="inlineStr">
@@ -20678,7 +20678,7 @@
       <c r="Q60" s="6" t="inlineStr"/>
       <c r="R60" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S60" s="6" t="inlineStr">
@@ -20772,7 +20772,7 @@
       <c r="Q61" s="6" t="inlineStr"/>
       <c r="R61" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S61" s="6" t="inlineStr">
@@ -20867,7 +20867,7 @@
       <c r="Q62" s="6" t="inlineStr"/>
       <c r="R62" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S62" s="6" t="inlineStr">
@@ -20961,7 +20961,7 @@
       <c r="Q63" s="6" t="inlineStr"/>
       <c r="R63" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S63" s="6" t="inlineStr">
@@ -21055,7 +21055,7 @@
       <c r="Q64" s="6" t="inlineStr"/>
       <c r="R64" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S64" s="6" t="inlineStr">
@@ -21149,7 +21149,7 @@
       <c r="Q65" s="6" t="inlineStr"/>
       <c r="R65" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S65" s="6" t="inlineStr">
@@ -21244,7 +21244,7 @@
       <c r="Q66" s="6" t="inlineStr"/>
       <c r="R66" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S66" s="6" t="inlineStr">
@@ -21339,7 +21339,7 @@
       <c r="Q67" s="6" t="inlineStr"/>
       <c r="R67" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S67" s="6" t="inlineStr">
@@ -21433,7 +21433,7 @@
       <c r="Q68" s="6" t="inlineStr"/>
       <c r="R68" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S68" s="6" t="inlineStr">
@@ -21528,7 +21528,7 @@
       <c r="Q69" s="6" t="inlineStr"/>
       <c r="R69" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S69" s="6" t="inlineStr">
@@ -21622,7 +21622,7 @@
       <c r="Q70" s="6" t="inlineStr"/>
       <c r="R70" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S70" s="6" t="inlineStr">
@@ -21716,7 +21716,7 @@
       <c r="Q71" s="6" t="inlineStr"/>
       <c r="R71" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S71" s="6" t="inlineStr">
@@ -21811,7 +21811,7 @@
       <c r="Q72" s="6" t="inlineStr"/>
       <c r="R72" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S72" s="6" t="inlineStr">
@@ -21905,7 +21905,7 @@
       <c r="Q73" s="6" t="inlineStr"/>
       <c r="R73" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S73" s="6" t="inlineStr">
@@ -22000,7 +22000,7 @@
       <c r="Q74" s="6" t="inlineStr"/>
       <c r="R74" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S74" s="6" t="inlineStr">
@@ -22095,7 +22095,7 @@
       <c r="Q75" s="6" t="inlineStr"/>
       <c r="R75" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S75" s="6" t="inlineStr">
@@ -22190,7 +22190,7 @@
       <c r="Q76" s="6" t="inlineStr"/>
       <c r="R76" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S76" s="6" t="inlineStr">
@@ -22285,7 +22285,7 @@
       <c r="Q77" s="6" t="inlineStr"/>
       <c r="R77" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S77" s="6" t="inlineStr">
@@ -22380,7 +22380,7 @@
       <c r="Q78" s="6" t="inlineStr"/>
       <c r="R78" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S78" s="6" t="inlineStr">
@@ -22475,7 +22475,7 @@
       <c r="Q79" s="6" t="inlineStr"/>
       <c r="R79" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S79" s="6" t="inlineStr">
@@ -22570,7 +22570,7 @@
       <c r="Q80" s="6" t="inlineStr"/>
       <c r="R80" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S80" s="6" t="inlineStr">
@@ -22664,7 +22664,7 @@
       <c r="Q81" s="6" t="inlineStr"/>
       <c r="R81" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S81" s="6" t="inlineStr">
@@ -22758,7 +22758,7 @@
       <c r="Q82" s="6" t="inlineStr"/>
       <c r="R82" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S82" s="6" t="inlineStr">
@@ -22852,7 +22852,7 @@
       <c r="Q83" s="6" t="inlineStr"/>
       <c r="R83" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S83" s="6" t="inlineStr">
@@ -22946,7 +22946,7 @@
       <c r="Q84" s="6" t="inlineStr"/>
       <c r="R84" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S84" s="6" t="inlineStr">
@@ -23040,7 +23040,7 @@
       <c r="Q85" s="6" t="inlineStr"/>
       <c r="R85" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S85" s="6" t="inlineStr">
@@ -23134,7 +23134,7 @@
       <c r="Q86" s="6" t="inlineStr"/>
       <c r="R86" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S86" s="6" t="inlineStr">
@@ -23230,7 +23230,7 @@
       <c r="Q87" s="6" t="inlineStr"/>
       <c r="R87" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S87" s="6" t="inlineStr">
@@ -23324,7 +23324,7 @@
       <c r="Q88" s="6" t="inlineStr"/>
       <c r="R88" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S88" s="6" t="inlineStr">
@@ -23419,7 +23419,7 @@
       <c r="Q89" s="6" t="inlineStr"/>
       <c r="R89" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S89" s="6" t="inlineStr">
@@ -23514,7 +23514,7 @@
       <c r="Q90" s="6" t="inlineStr"/>
       <c r="R90" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S90" s="6" t="inlineStr">
@@ -23609,7 +23609,7 @@
       <c r="Q91" s="6" t="inlineStr"/>
       <c r="R91" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S91" s="6" t="inlineStr">
@@ -23940,7 +23940,7 @@
       </c>
       <c r="R3" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S3" s="6" t="inlineStr">
@@ -24599,7 +24599,7 @@
       </c>
       <c r="R10" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S10" s="6" t="inlineStr">
@@ -24693,7 +24693,7 @@
       </c>
       <c r="R11" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S11" s="6" t="inlineStr">
@@ -28544,7 +28544,7 @@
       </c>
       <c r="R2" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S2" s="6" t="inlineStr">
@@ -28643,7 +28643,7 @@
       </c>
       <c r="R3" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S3" s="6" t="inlineStr">
@@ -28742,7 +28742,7 @@
       </c>
       <c r="R4" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S4" s="6" t="inlineStr">
@@ -28840,7 +28840,7 @@
       </c>
       <c r="R5" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S5" s="6" t="inlineStr">
@@ -31428,7 +31428,7 @@
       <c r="Q2" s="6" t="inlineStr"/>
       <c r="R2" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S2" s="6" t="inlineStr">
@@ -31522,7 +31522,7 @@
       <c r="Q3" s="6" t="inlineStr"/>
       <c r="R3" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S3" s="6" t="inlineStr">
@@ -31616,7 +31616,7 @@
       <c r="Q4" s="6" t="inlineStr"/>
       <c r="R4" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S4" s="6" t="inlineStr">
@@ -31710,7 +31710,7 @@
       <c r="Q5" s="6" t="inlineStr"/>
       <c r="R5" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S5" s="6" t="inlineStr">
@@ -31805,7 +31805,7 @@
       <c r="Q6" s="6" t="inlineStr"/>
       <c r="R6" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S6" s="6" t="inlineStr">
@@ -31899,7 +31899,7 @@
       <c r="Q7" s="6" t="inlineStr"/>
       <c r="R7" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S7" s="6" t="inlineStr">
@@ -31993,7 +31993,7 @@
       <c r="Q8" s="6" t="inlineStr"/>
       <c r="R8" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S8" s="6" t="inlineStr">
@@ -32087,7 +32087,7 @@
       <c r="Q9" s="6" t="inlineStr"/>
       <c r="R9" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S9" s="6" t="inlineStr">
@@ -32181,7 +32181,7 @@
       <c r="Q10" s="6" t="inlineStr"/>
       <c r="R10" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S10" s="6" t="inlineStr">
@@ -32275,7 +32275,7 @@
       <c r="Q11" s="6" t="inlineStr"/>
       <c r="R11" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S11" s="6" t="inlineStr">
@@ -32369,7 +32369,7 @@
       <c r="Q12" s="6" t="inlineStr"/>
       <c r="R12" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S12" s="6" t="inlineStr">
@@ -32463,7 +32463,7 @@
       <c r="Q13" s="6" t="inlineStr"/>
       <c r="R13" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S13" s="6" t="inlineStr">
@@ -32557,7 +32557,7 @@
       <c r="Q14" s="6" t="inlineStr"/>
       <c r="R14" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S14" s="6" t="inlineStr">
@@ -32651,7 +32651,7 @@
       <c r="Q15" s="6" t="inlineStr"/>
       <c r="R15" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S15" s="6" t="inlineStr">
@@ -32745,7 +32745,7 @@
       <c r="Q16" s="6" t="inlineStr"/>
       <c r="R16" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S16" s="6" t="inlineStr">
@@ -32839,7 +32839,7 @@
       <c r="Q17" s="6" t="inlineStr"/>
       <c r="R17" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S17" s="6" t="inlineStr">
@@ -32933,7 +32933,7 @@
       <c r="Q18" s="6" t="inlineStr"/>
       <c r="R18" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S18" s="6" t="inlineStr">
@@ -33027,7 +33027,7 @@
       <c r="Q19" s="6" t="inlineStr"/>
       <c r="R19" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S19" s="6" t="inlineStr">
@@ -33121,7 +33121,7 @@
       <c r="Q20" s="6" t="inlineStr"/>
       <c r="R20" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S20" s="6" t="inlineStr">
@@ -33216,7 +33216,7 @@
       <c r="Q21" s="6" t="inlineStr"/>
       <c r="R21" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S21" s="6" t="inlineStr">
@@ -33448,7 +33448,7 @@
       <c r="Q2" s="6" t="inlineStr"/>
       <c r="R2" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S2" s="6" t="inlineStr">
@@ -33542,7 +33542,7 @@
       <c r="Q3" s="6" t="inlineStr"/>
       <c r="R3" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S3" s="6" t="inlineStr">
@@ -33636,7 +33636,7 @@
       <c r="Q4" s="6" t="inlineStr"/>
       <c r="R4" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S4" s="6" t="inlineStr">
@@ -33730,7 +33730,7 @@
       <c r="Q5" s="6" t="inlineStr"/>
       <c r="R5" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S5" s="6" t="inlineStr">
@@ -33824,7 +33824,7 @@
       <c r="Q6" s="6" t="inlineStr"/>
       <c r="R6" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S6" s="6" t="inlineStr">
@@ -33918,7 +33918,7 @@
       <c r="Q7" s="6" t="inlineStr"/>
       <c r="R7" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S7" s="6" t="inlineStr">
@@ -34012,7 +34012,7 @@
       <c r="Q8" s="6" t="inlineStr"/>
       <c r="R8" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S8" s="6" t="inlineStr">
@@ -34106,7 +34106,7 @@
       <c r="Q9" s="6" t="inlineStr"/>
       <c r="R9" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S9" s="6" t="inlineStr">
@@ -34200,7 +34200,7 @@
       <c r="Q10" s="6" t="inlineStr"/>
       <c r="R10" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S10" s="6" t="inlineStr">
@@ -34294,7 +34294,7 @@
       <c r="Q11" s="6" t="inlineStr"/>
       <c r="R11" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S11" s="6" t="inlineStr">
@@ -34388,7 +34388,7 @@
       <c r="Q12" s="6" t="inlineStr"/>
       <c r="R12" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S12" s="6" t="inlineStr">
@@ -34482,7 +34482,7 @@
       <c r="Q13" s="6" t="inlineStr"/>
       <c r="R13" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S13" s="6" t="inlineStr">
@@ -34576,7 +34576,7 @@
       <c r="Q14" s="6" t="inlineStr"/>
       <c r="R14" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S14" s="6" t="inlineStr">
@@ -34670,7 +34670,7 @@
       <c r="Q15" s="6" t="inlineStr"/>
       <c r="R15" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S15" s="6" t="inlineStr">
@@ -34764,7 +34764,7 @@
       <c r="Q16" s="6" t="inlineStr"/>
       <c r="R16" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S16" s="6" t="inlineStr">
@@ -34858,7 +34858,7 @@
       <c r="Q17" s="6" t="inlineStr"/>
       <c r="R17" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S17" s="6" t="inlineStr">
@@ -34952,7 +34952,7 @@
       <c r="Q18" s="6" t="inlineStr"/>
       <c r="R18" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S18" s="6" t="inlineStr">
@@ -35046,7 +35046,7 @@
       <c r="Q19" s="6" t="inlineStr"/>
       <c r="R19" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S19" s="6" t="inlineStr">
@@ -35140,7 +35140,7 @@
       <c r="Q20" s="6" t="inlineStr"/>
       <c r="R20" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S20" s="6" t="inlineStr">
@@ -35234,7 +35234,7 @@
       <c r="Q21" s="6" t="inlineStr"/>
       <c r="R21" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S21" s="6" t="inlineStr">
@@ -35328,7 +35328,7 @@
       <c r="Q22" s="6" t="inlineStr"/>
       <c r="R22" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S22" s="6" t="inlineStr">
@@ -35422,7 +35422,7 @@
       <c r="Q23" s="6" t="inlineStr"/>
       <c r="R23" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S23" s="6" t="inlineStr">
@@ -35516,7 +35516,7 @@
       <c r="Q24" s="6" t="inlineStr"/>
       <c r="R24" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S24" s="6" t="inlineStr">
@@ -35610,7 +35610,7 @@
       <c r="Q25" s="6" t="inlineStr"/>
       <c r="R25" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S25" s="6" t="inlineStr">
@@ -35704,7 +35704,7 @@
       <c r="Q26" s="6" t="inlineStr"/>
       <c r="R26" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S26" s="6" t="inlineStr">
@@ -35798,7 +35798,7 @@
       <c r="Q27" s="6" t="inlineStr"/>
       <c r="R27" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S27" s="6" t="inlineStr">
@@ -35892,7 +35892,7 @@
       <c r="Q28" s="6" t="inlineStr"/>
       <c r="R28" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S28" s="6" t="inlineStr">
@@ -35986,7 +35986,7 @@
       <c r="Q29" s="6" t="inlineStr"/>
       <c r="R29" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S29" s="6" t="inlineStr">
@@ -36080,7 +36080,7 @@
       <c r="Q30" s="6" t="inlineStr"/>
       <c r="R30" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S30" s="6" t="inlineStr">
@@ -36174,7 +36174,7 @@
       <c r="Q31" s="6" t="inlineStr"/>
       <c r="R31" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S31" s="6" t="inlineStr">
@@ -36268,7 +36268,7 @@
       <c r="Q32" s="6" t="inlineStr"/>
       <c r="R32" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S32" s="6" t="inlineStr">
@@ -36362,7 +36362,7 @@
       <c r="Q33" s="6" t="inlineStr"/>
       <c r="R33" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S33" s="6" t="inlineStr">
@@ -36456,7 +36456,7 @@
       <c r="Q34" s="6" t="inlineStr"/>
       <c r="R34" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S34" s="6" t="inlineStr">
@@ -36550,7 +36550,7 @@
       <c r="Q35" s="6" t="inlineStr"/>
       <c r="R35" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S35" s="6" t="inlineStr">
@@ -36644,7 +36644,7 @@
       <c r="Q36" s="6" t="inlineStr"/>
       <c r="R36" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S36" s="6" t="inlineStr">
@@ -36738,7 +36738,7 @@
       <c r="Q37" s="6" t="inlineStr"/>
       <c r="R37" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S37" s="6" t="inlineStr">
@@ -36832,7 +36832,7 @@
       <c r="Q38" s="6" t="inlineStr"/>
       <c r="R38" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S38" s="6" t="inlineStr">
@@ -36926,7 +36926,7 @@
       <c r="Q39" s="6" t="inlineStr"/>
       <c r="R39" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S39" s="6" t="inlineStr">
@@ -37020,7 +37020,7 @@
       <c r="Q40" s="6" t="inlineStr"/>
       <c r="R40" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S40" s="6" t="inlineStr">
@@ -37114,7 +37114,7 @@
       <c r="Q41" s="6" t="inlineStr"/>
       <c r="R41" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S41" s="6" t="inlineStr">
@@ -37208,7 +37208,7 @@
       <c r="Q42" s="6" t="inlineStr"/>
       <c r="R42" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S42" s="6" t="inlineStr">
@@ -37302,7 +37302,7 @@
       <c r="Q43" s="6" t="inlineStr"/>
       <c r="R43" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S43" s="6" t="inlineStr">
@@ -37396,7 +37396,7 @@
       <c r="Q44" s="6" t="inlineStr"/>
       <c r="R44" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S44" s="6" t="inlineStr">
@@ -37491,7 +37491,7 @@
       <c r="Q45" s="6" t="inlineStr"/>
       <c r="R45" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S45" s="6" t="inlineStr">
@@ -37585,7 +37585,7 @@
       <c r="Q46" s="6" t="inlineStr"/>
       <c r="R46" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S46" s="6" t="inlineStr">
@@ -37679,7 +37679,7 @@
       <c r="Q47" s="6" t="inlineStr"/>
       <c r="R47" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S47" s="6" t="inlineStr">
@@ -37773,7 +37773,7 @@
       <c r="Q48" s="6" t="inlineStr"/>
       <c r="R48" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S48" s="6" t="inlineStr">
@@ -37867,7 +37867,7 @@
       <c r="Q49" s="6" t="inlineStr"/>
       <c r="R49" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S49" s="6" t="inlineStr">
@@ -37961,7 +37961,7 @@
       <c r="Q50" s="6" t="inlineStr"/>
       <c r="R50" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S50" s="6" t="inlineStr">
@@ -38056,7 +38056,7 @@
       <c r="Q51" s="6" t="inlineStr"/>
       <c r="R51" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S51" s="6" t="inlineStr">
@@ -38151,7 +38151,7 @@
       <c r="Q52" s="6" t="inlineStr"/>
       <c r="R52" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S52" s="6" t="inlineStr">
@@ -38245,7 +38245,7 @@
       <c r="Q53" s="6" t="inlineStr"/>
       <c r="R53" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S53" s="6" t="inlineStr">
@@ -38339,7 +38339,7 @@
       <c r="Q54" s="6" t="inlineStr"/>
       <c r="R54" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S54" s="6" t="inlineStr">
@@ -38433,7 +38433,7 @@
       <c r="Q55" s="6" t="inlineStr"/>
       <c r="R55" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S55" s="6" t="inlineStr">
@@ -38527,7 +38527,7 @@
       <c r="Q56" s="6" t="inlineStr"/>
       <c r="R56" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S56" s="6" t="inlineStr">
@@ -38621,7 +38621,7 @@
       <c r="Q57" s="6" t="inlineStr"/>
       <c r="R57" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S57" s="6" t="inlineStr">
@@ -38715,7 +38715,7 @@
       <c r="Q58" s="6" t="inlineStr"/>
       <c r="R58" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S58" s="6" t="inlineStr">
@@ -38809,7 +38809,7 @@
       <c r="Q59" s="6" t="inlineStr"/>
       <c r="R59" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S59" s="6" t="inlineStr">
@@ -39047,7 +39047,7 @@
       </c>
       <c r="R2" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S2" s="6" t="inlineStr">
@@ -39142,7 +39142,7 @@
       </c>
       <c r="R3" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S3" s="6" t="inlineStr">
@@ -39237,7 +39237,7 @@
       </c>
       <c r="R4" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="S4" s="6" t="inlineStr">

</xml_diff>